<commit_message>
Remove estimated costs from ZT411 comparison; add stock and contact rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ldo83LUj559GT8miB72wwC
</commit_message>
<xml_diff>
--- a/ZT411_300dpi_헤드_업체비교.xlsx
+++ b/ZT411_300dpi_헤드_업체비교.xlsx
@@ -113,7 +113,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D21" authorId="0">
+    <comment ref="D23" authorId="0">
       <text>
         <r>
           <rPr>
@@ -121,7 +121,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">추정값</t>
+          <t xml:space="preserve">업체 운임 견적 받으면 입력 </t>
         </r>
         <r>
           <rPr>
@@ -129,7 +129,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">($80): </t>
+          <t xml:space="preserve">(EXW: </t>
         </r>
         <r>
           <rPr>
@@ -137,7 +137,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">헤드 </t>
+          <t xml:space="preserve">중국 내 픽업</t>
         </r>
         <r>
           <rPr>
@@ -145,7 +145,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">·</t>
         </r>
         <r>
           <rPr>
@@ -153,7 +153,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">개</t>
+          <t xml:space="preserve">수출통관 비용 포함 여부 확인</t>
         </r>
         <r>
           <rPr>
@@ -161,171 +161,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">(</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">약 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">3~5kg) </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">중국→한국 특송 기준 대략치</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">. EXW </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">조건이라 중국 내 픽업</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">·</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">수출통관 비용이 추가될 수 있음</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">. </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">업체 운임 견적 받으면 수정</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D24" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">프린터 부품</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">(HS 8443.99)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">은 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">ITA </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">품목으로 기본관세 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">0%</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">로 추정</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">. </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">관세사 확인 필요</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">.</t>
+          <t xml:space="preserve">)</t>
         </r>
       </text>
     </comment>
@@ -337,7 +173,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">부가세 </t>
+          <t xml:space="preserve">관세사 확인 후 입력 </t>
         </r>
         <r>
           <rPr>
@@ -345,7 +181,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">= (</t>
+          <t xml:space="preserve">(</t>
         </r>
         <r>
           <rPr>
@@ -353,7 +189,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">과세가격 </t>
+          <t xml:space="preserve">예</t>
         </r>
         <r>
           <rPr>
@@ -361,7 +197,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">+ </t>
+          <t xml:space="preserve">: 0%</t>
         </r>
         <r>
           <rPr>
@@ -369,7 +205,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">관세</t>
+          <t xml:space="preserve">면 </t>
         </r>
         <r>
           <rPr>
@@ -377,7 +213,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">) × 10%. </t>
+          <t xml:space="preserve">0 </t>
         </r>
         <r>
           <rPr>
@@ -385,99 +221,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">사업자 매입세액 공제</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">(</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">환급</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">) </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">가능</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D27" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">추정값</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">: </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">특송 통관수수료</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">·</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">관세사 수수료 등 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">(</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">실제 청구액으로 수정</t>
+          <t xml:space="preserve">입력</t>
         </r>
         <r>
           <rPr>
@@ -497,7 +241,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">추정값</t>
+          <t xml:space="preserve">부가세 </t>
         </r>
         <r>
           <rPr>
@@ -505,7 +249,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: T/T </t>
+          <t xml:space="preserve">= (</t>
         </r>
         <r>
           <rPr>
@@ -513,7 +257,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">해외송금 수수료</t>
+          <t xml:space="preserve">과세가격 </t>
         </r>
         <r>
           <rPr>
@@ -521,7 +265,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">+</t>
+          <t xml:space="preserve">+ </t>
         </r>
         <r>
           <rPr>
@@ -529,7 +273,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">전신료 </t>
+          <t xml:space="preserve">관세</t>
         </r>
         <r>
           <rPr>
@@ -537,6 +281,22 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">) × 10%. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">사업자 매입세액 공제</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">(</t>
         </r>
         <r>
@@ -545,7 +305,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">은행별 상이</t>
+          <t xml:space="preserve">환급</t>
         </r>
         <r>
           <rPr>
@@ -553,11 +313,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">)</t>
+          <t xml:space="preserve">) </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">가능</t>
         </r>
       </text>
     </comment>
-    <comment ref="E21" authorId="0">
+    <comment ref="D29" authorId="0">
       <text>
         <r>
           <rPr>
@@ -565,7 +333,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">추정값</t>
+          <t xml:space="preserve">실제 청구액 입력 </t>
         </r>
         <r>
           <rPr>
@@ -573,7 +341,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">($80). FOB </t>
+          <t xml:space="preserve">(</t>
         </r>
         <r>
           <rPr>
@@ -581,6 +349,62 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">특송 통관수수료</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">·</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">관세사 수수료 등</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D30" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">실제 송금 수수료 입력</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">FOB </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">조건 — </t>
         </r>
         <r>
@@ -613,7 +437,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">견적 받으면 수정</t>
+          <t xml:space="preserve">받으면 입력</t>
         </r>
         <r>
           <rPr>
@@ -669,7 +493,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F21" authorId="0">
+    <comment ref="F23" authorId="0">
       <text>
         <r>
           <rPr>
@@ -677,7 +501,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">추정값</t>
+          <t xml:space="preserve">업체 운임 견적 받으면 입력 </t>
         </r>
         <r>
           <rPr>
@@ -685,7 +509,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">($80). EXW </t>
+          <t xml:space="preserve">(EXW </t>
         </r>
         <r>
           <rPr>
@@ -693,7 +517,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">조건 — 중국 내 픽업</t>
+          <t xml:space="preserve">조건</t>
         </r>
         <r>
           <rPr>
@@ -701,39 +525,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">·</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">수출통관 비용 추가 가능</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">. </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">견적 받으면 수정</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">.</t>
+          <t xml:space="preserve">)</t>
         </r>
       </text>
     </comment>
@@ -742,7 +534,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="71">
   <si>
     <r>
       <rPr>
@@ -1816,6 +1608,120 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">재고여부</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미확인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결제 후 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일 이내 출고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">미확인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">담당자</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미기재 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Guangzhou ASON </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명의로 소개</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Jason Chen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon Li (Simo)</t>
+  </si>
+  <si>
     <t xml:space="preserve">비고</t>
   </si>
   <si>
@@ -3433,7 +3339,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">총 비용의 노란 셀</t>
+      <t xml:space="preserve">총 비용의 노란 빈칸</t>
     </r>
     <r>
       <rPr>
@@ -3501,7 +3407,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">은 추정값 → 업체 운임 견적</t>
+      <t xml:space="preserve">은 미확정 → 확인되는 대로 입력하면 총 비용 자동 재계산 </t>
     </r>
     <r>
       <rPr>
@@ -3510,15 +3416,41 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">실제 청구액으로 수정하면 자동 재계산</t>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빈칸은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">으로 계산됨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -4247,7 +4179,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:F47"/>
+  <dimension ref="B2:F49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -4453,361 +4385,369 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C16" s="15"/>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="17" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="17" t="s">
         <v>35</v>
       </c>
       <c r="F16" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="9" t="s">
         <v>36</v>
       </c>
+      <c r="C17" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
+    <row r="18" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="s">
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C21" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D21" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F21" s="8" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="20" t="n">
-        <f aca="false">D7*D9</f>
-        <v>2400</v>
-      </c>
-      <c r="E20" s="20" t="n">
-        <f aca="false">E7*E9</f>
-        <v>2800</v>
-      </c>
-      <c r="F20" s="20" t="n">
-        <f aca="false">F7*F9</f>
-        <v>2700</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="11" t="n">
-        <v>80</v>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>80</v>
-      </c>
-      <c r="F21" s="11" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D22" s="20" t="n">
-        <f aca="false">D20+D21</f>
-        <v>2480</v>
+        <f aca="false">D7*D9</f>
+        <v>2400</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">E20+E21</f>
-        <v>2880</v>
+        <f aca="false">E7*E9</f>
+        <v>2800</v>
       </c>
       <c r="F22" s="20" t="n">
-        <f aca="false">F20+F21</f>
-        <v>2780</v>
+        <f aca="false">F7*F9</f>
+        <v>2700</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C23" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="13" t="n">
-        <f aca="false">D22*$D$2</f>
-        <v>3376520</v>
-      </c>
-      <c r="E23" s="13" t="n">
-        <f aca="false">E22*$D$2</f>
-        <v>3921120</v>
-      </c>
-      <c r="F23" s="13" t="n">
-        <f aca="false">F22*$D$2</f>
-        <v>3784970</v>
-      </c>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C24" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="21" t="n">
-        <v>0</v>
+      <c r="D24" s="20" t="n">
+        <f aca="false">D22+D23</f>
+        <v>2400</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <f aca="false">E22+E23</f>
+        <v>2800</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <f aca="false">F22+F23</f>
+        <v>2700</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="13" t="n">
-        <f aca="false">ROUND(D23*D24,0)</f>
-        <v>0</v>
+        <f aca="false">D24*$D$2</f>
+        <v>3267600</v>
       </c>
       <c r="E25" s="13" t="n">
-        <f aca="false">ROUND(E23*E24,0)</f>
-        <v>0</v>
+        <f aca="false">E24*$D$2</f>
+        <v>3812200</v>
       </c>
       <c r="F25" s="13" t="n">
-        <f aca="false">ROUND(F23*F24,0)</f>
-        <v>0</v>
+        <f aca="false">F24*$D$2</f>
+        <v>3676050</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="13" t="n">
-        <f aca="false">ROUND((D23+D25)*0.1,0)</f>
-        <v>337652</v>
-      </c>
-      <c r="E26" s="13" t="n">
-        <f aca="false">ROUND((E23+E25)*0.1,0)</f>
-        <v>392112</v>
-      </c>
-      <c r="F26" s="13" t="n">
-        <f aca="false">ROUND((F23+F25)*0.1,0)</f>
-        <v>378497</v>
-      </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="12" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E27" s="12" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F27" s="12" t="n">
-        <v>30000</v>
+      <c r="D27" s="13" t="n">
+        <f aca="false">ROUND(D25*D26,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <f aca="false">ROUND(E25*E26,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="13" t="n">
+        <f aca="false">ROUND(F25*F26,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="E28" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F28" s="12" t="n">
-        <v>20000</v>
+      <c r="D28" s="13" t="n">
+        <f aca="false">ROUND((D25+D27)*0.1,0)</f>
+        <v>326760</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <f aca="false">ROUND((E25+E27)*0.1,0)</f>
+        <v>381220</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <f aca="false">ROUND((F25+F27)*0.1,0)</f>
+        <v>367605</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" s="19" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="D29" s="23" t="n">
-        <f aca="false">D23+D25+D26+D27+D28</f>
-        <v>3764172</v>
-      </c>
-      <c r="E29" s="23" t="n">
-        <f aca="false">E23+E25+E26+E27+E28</f>
-        <v>4363232</v>
-      </c>
-      <c r="F29" s="23" t="n">
-        <f aca="false">F23+F25+F26+F27+F28</f>
-        <v>4213467</v>
-      </c>
+      <c r="B29" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C30" s="19" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <f aca="false">ROUND(D29/D9,0)</f>
-        <v>376417</v>
-      </c>
-      <c r="E30" s="13" t="n">
-        <f aca="false">ROUND(E29/E9,0)</f>
-        <v>436323</v>
-      </c>
-      <c r="F30" s="13" t="n">
-        <f aca="false">ROUND(F29/F9,0)</f>
-        <v>421347</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="9" t="s">
-        <v>49</v>
+      <c r="B31" s="22" t="s">
+        <v>54</v>
       </c>
       <c r="C31" s="19" t="str">
         <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
         <v>-</v>
       </c>
-      <c r="D31" s="13" t="n">
-        <f aca="false">D29-D26</f>
-        <v>3426520</v>
-      </c>
-      <c r="E31" s="13" t="n">
-        <f aca="false">E29-E26</f>
-        <v>3971120</v>
-      </c>
-      <c r="F31" s="13" t="n">
-        <f aca="false">F29-F26</f>
-        <v>3834970</v>
+      <c r="D31" s="23" t="n">
+        <f aca="false">D25+D27+D28+D29+D30</f>
+        <v>3594360</v>
+      </c>
+      <c r="E31" s="23" t="n">
+        <f aca="false">E25+E27+E28+E29+E30</f>
+        <v>4193420</v>
+      </c>
+      <c r="F31" s="23" t="n">
+        <f aca="false">F25+F27+F28+F29+F30</f>
+        <v>4043655</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C32" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="19" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D32" s="13" t="n">
+        <f aca="false">ROUND(D31/D9,0)</f>
+        <v>359436</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <f aca="false">ROUND(E31/E9,0)</f>
+        <v>419342</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <f aca="false">ROUND(F31/F9,0)</f>
+        <v>404366</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" s="19" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D33" s="13" t="n">
+        <f aca="false">D31-D28</f>
+        <v>3267600</v>
+      </c>
+      <c r="E33" s="13" t="n">
+        <f aca="false">E31-E28</f>
+        <v>3812200</v>
+      </c>
+      <c r="F33" s="13" t="n">
+        <f aca="false">F31-F28</f>
+        <v>3676050</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D32" s="13" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*D9-D31,"국내단가 입력 필요")</f>
+      <c r="D34" s="13" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*D9-D33,"국내단가 입력 필요")</f>
         <v>국내단가 입력 필요</v>
       </c>
-      <c r="E32" s="13" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*E9-E31,"국내단가 입력 필요")</f>
+      <c r="E34" s="13" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*E9-E33,"국내단가 입력 필요")</f>
         <v>국내단가 입력 필요</v>
       </c>
-      <c r="F32" s="13" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*F9-F31,"국내단가 입력 필요")</f>
+      <c r="F34" s="13" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*F9-F33,"국내단가 입력 필요")</f>
         <v>국내단가 입력 필요</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="24" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="25" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="25" t="s">
-        <v>53</v>
+      <c r="B36" s="24" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="25" t="s">
-        <v>54</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="25" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="24" t="s">
-        <v>55</v>
+      <c r="B39" s="25" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="25" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="25" t="s">
-        <v>57</v>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="25" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="25" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="25" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="25" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="25" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="25" t="s">
-        <v>63</v>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B48" s="25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="25" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -4821,9 +4761,9 @@
       <formula>D8=MIN($D$8:$F$8)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D29:F29">
+  <conditionalFormatting sqref="D31:F31">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>D29=MIN($D$29:$F$29)</formula>
+      <formula>D31=MIN($D$31:$F$31)</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Remove stock row from ZT411 comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ldo83LUj559GT8miB72wwC
</commit_message>
<xml_diff>
--- a/ZT411_300dpi_헤드_업체비교.xlsx
+++ b/ZT411_300dpi_헤드_업체비교.xlsx
@@ -113,7 +113,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0">
+    <comment ref="D22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -165,7 +165,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D26" authorId="0">
+    <comment ref="D25" authorId="0">
       <text>
         <r>
           <rPr>
@@ -230,6 +230,98 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D27" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">부가세 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">= (</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">과세가격 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">+ </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">관세</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">) × 10%. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">사업자 매입세액 공제</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">환급</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">) </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">가능</t>
         </r>
       </text>
     </comment>
@@ -241,7 +333,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">부가세 </t>
+          <t xml:space="preserve">실제 청구액 입력 </t>
         </r>
         <r>
           <rPr>
@@ -249,7 +341,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">= (</t>
+          <t xml:space="preserve">(</t>
         </r>
         <r>
           <rPr>
@@ -257,7 +349,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">과세가격 </t>
+          <t xml:space="preserve">특송 통관수수료</t>
         </r>
         <r>
           <rPr>
@@ -265,7 +357,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">+ </t>
+          <t xml:space="preserve">·</t>
         </r>
         <r>
           <rPr>
@@ -273,7 +365,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">관세</t>
+          <t xml:space="preserve">관세사 수수료 등</t>
         </r>
         <r>
           <rPr>
@@ -281,47 +373,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">) × 10%. </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">사업자 매입세액 공제</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">(</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">환급</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">) </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">가능</t>
+          <t xml:space="preserve">)</t>
         </r>
       </text>
     </comment>
@@ -333,63 +385,11 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">실제 청구액 입력 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">(</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">특송 통관수수료</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">·</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">관세사 수수료 등</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">)</t>
+          <t xml:space="preserve">실제 송금 수수료 입력</t>
         </r>
       </text>
     </comment>
-    <comment ref="D30" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">실제 송금 수수료 입력</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E23" authorId="0">
+    <comment ref="E22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -493,7 +493,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F23" authorId="0">
+    <comment ref="F22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -534,7 +534,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="68">
   <si>
     <r>
       <rPr>
@@ -1606,71 +1606,6 @@
       </rPr>
       <t xml:space="preserve">O</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">재고여부</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">미확인 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">결제 후 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일 이내 출고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">미확인</t>
   </si>
   <si>
     <t xml:space="preserve">담당자</t>
@@ -4179,7 +4114,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:F49"/>
+  <dimension ref="B2:F48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -4389,200 +4324,196 @@
       <c r="B16" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="15"/>
+      <c r="C16" s="15" t="s">
+        <v>10</v>
+      </c>
       <c r="D16" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="17" t="s">
-        <v>35</v>
+      <c r="F16" s="16" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="F18" s="17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>8</v>
+      <c r="D21" s="20" t="n">
+        <f aca="false">D7*D9</f>
+        <v>2400</v>
+      </c>
+      <c r="E21" s="20" t="n">
+        <f aca="false">E7*E9</f>
+        <v>2800</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <f aca="false">F7*F9</f>
+        <v>2700</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D22" s="20" t="n">
-        <f aca="false">D7*D9</f>
-        <v>2400</v>
-      </c>
-      <c r="E22" s="20" t="n">
-        <f aca="false">E7*E9</f>
-        <v>2800</v>
-      </c>
-      <c r="F22" s="20" t="n">
-        <f aca="false">F7*F9</f>
-        <v>2700</v>
-      </c>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C23" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
+      <c r="D23" s="20" t="n">
+        <f aca="false">D21+D22</f>
+        <v>2400</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <f aca="false">E21+E22</f>
+        <v>2800</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <f aca="false">F21+F22</f>
+        <v>2700</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C24" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="20" t="n">
-        <f aca="false">D22+D23</f>
-        <v>2400</v>
-      </c>
-      <c r="E24" s="20" t="n">
-        <f aca="false">E22+E23</f>
-        <v>2800</v>
-      </c>
-      <c r="F24" s="20" t="n">
-        <f aca="false">F22+F23</f>
-        <v>2700</v>
+      <c r="D24" s="13" t="n">
+        <f aca="false">D23*$D$2</f>
+        <v>3267600</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <f aca="false">E23*$D$2</f>
+        <v>3812200</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <f aca="false">F23*$D$2</f>
+        <v>3676050</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="13" t="n">
-        <f aca="false">D24*$D$2</f>
-        <v>3267600</v>
-      </c>
-      <c r="E25" s="13" t="n">
-        <f aca="false">E24*$D$2</f>
-        <v>3812200</v>
-      </c>
-      <c r="F25" s="13" t="n">
-        <f aca="false">F24*$D$2</f>
-        <v>3676050</v>
-      </c>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
+      <c r="D26" s="13" t="n">
+        <f aca="false">ROUND(D24*D25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <f aca="false">ROUND(E24*E25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <f aca="false">ROUND(F24*F25,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="13" t="n">
-        <f aca="false">ROUND(D25*D26,0)</f>
-        <v>0</v>
+        <f aca="false">ROUND((D24+D26)*0.1,0)</f>
+        <v>326760</v>
       </c>
       <c r="E27" s="13" t="n">
-        <f aca="false">ROUND(E25*E26,0)</f>
-        <v>0</v>
+        <f aca="false">ROUND((E24+E26)*0.1,0)</f>
+        <v>381220</v>
       </c>
       <c r="F27" s="13" t="n">
-        <f aca="false">ROUND(F25*F26,0)</f>
-        <v>0</v>
+        <f aca="false">ROUND((F24+F26)*0.1,0)</f>
+        <v>367605</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="13" t="n">
-        <f aca="false">ROUND((D25+D27)*0.1,0)</f>
-        <v>326760</v>
-      </c>
-      <c r="E28" s="13" t="n">
-        <f aca="false">ROUND((E25+E27)*0.1,0)</f>
-        <v>381220</v>
-      </c>
-      <c r="F28" s="13" t="n">
-        <f aca="false">ROUND((F25+F27)*0.1,0)</f>
-        <v>367605</v>
-      </c>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C29" s="19" t="s">
         <v>10</v>
@@ -4592,162 +4523,151 @@
       <c r="F29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
+      <c r="B30" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="19" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D30" s="23" t="n">
+        <f aca="false">D24+D26+D27+D28+D29</f>
+        <v>3594360</v>
+      </c>
+      <c r="E30" s="23" t="n">
+        <f aca="false">E24+E26+E27+E28+E29</f>
+        <v>4193420</v>
+      </c>
+      <c r="F30" s="23" t="n">
+        <f aca="false">F24+F26+F27+F28+F29</f>
+        <v>4043655</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="22" t="s">
-        <v>54</v>
+      <c r="B31" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="C31" s="19" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
+        <f aca="false">IF(ISNUMBER($C$8),$C$8,"-")</f>
         <v>-</v>
       </c>
-      <c r="D31" s="23" t="n">
-        <f aca="false">D25+D27+D28+D29+D30</f>
-        <v>3594360</v>
-      </c>
-      <c r="E31" s="23" t="n">
-        <f aca="false">E25+E27+E28+E29+E30</f>
-        <v>4193420</v>
-      </c>
-      <c r="F31" s="23" t="n">
-        <f aca="false">F25+F27+F28+F29+F30</f>
-        <v>4043655</v>
+      <c r="D31" s="13" t="n">
+        <f aca="false">ROUND(D30/D9,0)</f>
+        <v>359436</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <f aca="false">ROUND(E30/E9,0)</f>
+        <v>419342</v>
+      </c>
+      <c r="F31" s="13" t="n">
+        <f aca="false">ROUND(F30/F9,0)</f>
+        <v>404366</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C32" s="19" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8,"-")</f>
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
         <v>-</v>
       </c>
       <c r="D32" s="13" t="n">
-        <f aca="false">ROUND(D31/D9,0)</f>
-        <v>359436</v>
+        <f aca="false">D30-D27</f>
+        <v>3267600</v>
       </c>
       <c r="E32" s="13" t="n">
-        <f aca="false">ROUND(E31/E9,0)</f>
-        <v>419342</v>
+        <f aca="false">E30-E27</f>
+        <v>3812200</v>
       </c>
       <c r="F32" s="13" t="n">
-        <f aca="false">ROUND(F31/F9,0)</f>
-        <v>404366</v>
+        <f aca="false">F30-F27</f>
+        <v>3676050</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="19" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*10,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <f aca="false">D31-D28</f>
-        <v>3267600</v>
-      </c>
-      <c r="E33" s="13" t="n">
-        <f aca="false">E31-E28</f>
-        <v>3812200</v>
-      </c>
-      <c r="F33" s="13" t="n">
-        <f aca="false">F31-F28</f>
-        <v>3676050</v>
+        <v>54</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="13" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*D9-D32,"국내단가 입력 필요")</f>
+        <v>국내단가 입력 필요</v>
+      </c>
+      <c r="E33" s="13" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*E9-E32,"국내단가 입력 필요")</f>
+        <v>국내단가 입력 필요</v>
+      </c>
+      <c r="F33" s="13" t="str">
+        <f aca="false">IF(ISNUMBER($C$8),$C$8*F9-F32,"국내단가 입력 필요")</f>
+        <v>국내단가 입력 필요</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" s="13" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*D9-D33,"국내단가 입력 필요")</f>
-        <v>국내단가 입력 필요</v>
-      </c>
-      <c r="E34" s="13" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*E9-E33,"국내단가 입력 필요")</f>
-        <v>국내단가 입력 필요</v>
-      </c>
-      <c r="F34" s="13" t="str">
-        <f aca="false">IF(ISNUMBER($C$8),$C$8*F9-F33,"국내단가 입력 필요")</f>
-        <v>국내단가 입력 필요</v>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="24" t="s">
-        <v>58</v>
+      <c r="B36" s="25" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="25" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="25" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="25" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="24" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="25" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="25" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="25" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="25" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -4761,9 +4681,9 @@
       <formula>D8=MIN($D$8:$F$8)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D31:F31">
+  <conditionalFormatting sqref="D30:F30">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>D31=MIN($D$31:$F$31)</formula>
+      <formula>D30=MIN($D$30:$F$30)</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>